<commit_message>
Autosize Excel columns so headers and values fit
Widen sheet columns based on label and sample cell length for the
daily and period CBPOL workbooks.

Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/cbpol_taxas_acumuladas_periodos.xlsx
+++ b/output/cbpol_taxas_acumuladas_periodos.xlsx
@@ -422,6 +422,10 @@
   </sheetPr>
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -532,6 +536,13 @@
   </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -723,6 +734,14 @@
   </sheetPr>
   <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2064,6 +2083,14 @@
   </sheetPr>
   <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3237,6 +3264,14 @@
   </sheetPr>
   <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4410,6 +4445,14 @@
   </sheetPr>
   <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5583,6 +5626,14 @@
   </sheetPr>
   <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6728,6 +6779,14 @@
   </sheetPr>
   <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>